<commit_message>
samples(lem): problem 16's rapid-drawdown dam sits on El. 182, the same base as problem 8
xslope_gsat_rapid.xlsx carried an entered Max depth of 0 where the four other
files for this dam have 182. The file now has a builder
(benchmarks/build_lem_samples.py) that reads problem 8's workbook and adds only
problem 16's saturated unit weights and post-drawdown line, so the dam cannot
drift again; verify_rebuild gains a lem_samples group. Bishop 1.120 and Spencer
1.121 are unchanged: the governing circle is tangent at El. 197 and never
reached either base. Results figure and the template-docs sheet images redrawn;
corpus index regenerated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/usage/sample_sheets/sheets_rapid.xlsx
+++ b/docs/usage/sample_sheets/sheets_rapid.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/.claude/worktrees/joints-r1/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E12967D2-A998-D342-B5ED-43CABE326A3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{119A1861-00BF-3949-902B-66F34C8769AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15680" yWindow="4780" windowWidth="46940" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4280" yWindow="2000" windowWidth="40460" windowHeight="22500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -23,11 +23,12 @@
     <sheet name="dloads" sheetId="8" r:id="rId8"/>
     <sheet name="dloads (2)" sheetId="9" r:id="rId9"/>
     <sheet name="reinforce" sheetId="10" r:id="rId10"/>
-    <sheet name="piles" sheetId="11" r:id="rId11"/>
-    <sheet name="lloads" sheetId="12" r:id="rId12"/>
-    <sheet name="seep bc" sheetId="13" r:id="rId13"/>
-    <sheet name="seep bc (2)" sheetId="14" r:id="rId14"/>
-    <sheet name="tseep" sheetId="15" r:id="rId15"/>
+    <sheet name="joints" sheetId="16" r:id="rId11"/>
+    <sheet name="piles" sheetId="11" r:id="rId12"/>
+    <sheet name="lloads" sheetId="12" r:id="rId13"/>
+    <sheet name="seep bc" sheetId="13" r:id="rId14"/>
+    <sheet name="seep bc (2)" sheetId="14" r:id="rId15"/>
+    <sheet name="tseep" sheetId="15" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="crack_depth">main!$D$11</definedName>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="329">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -1137,6 +1138,36 @@
   </si>
   <si>
     <t>l</t>
+  </si>
+  <si>
+    <t>Joint</t>
+  </si>
+  <si>
+    <t>kn</t>
+  </si>
+  <si>
+    <t>ks</t>
+  </si>
+  <si>
+    <t>Jred</t>
+  </si>
+  <si>
+    <t>phi</t>
+  </si>
+  <si>
+    <t>joints</t>
+  </si>
+  <si>
+    <t>Slip joints (interfaces with no reinforcement)</t>
+  </si>
+  <si>
+    <t>c_res</t>
+  </si>
+  <si>
+    <t>phi_res</t>
+  </si>
+  <si>
+    <t>dil</t>
   </si>
 </sst>
 </file>
@@ -1644,7 +1675,21 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="35">
+  <dxfs count="37">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1907,16 +1952,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>217714</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>54430</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>326571</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>9073</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
-      <xdr:colOff>444500</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>90714</xdr:rowOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>553357</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>172358</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1931,8 +1976,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16455571" y="254001"/>
-          <a:ext cx="3855358" cy="4027713"/>
+          <a:off x="19866428" y="1006930"/>
+          <a:ext cx="3855358" cy="4753428"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2060,7 +2105,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0"/>
-            <a:t> = soii-reinforcement interface adhesion (blank</a:t>
+            <a:t> = soil-reinforcement interface adhesion (blank</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
@@ -2105,7 +2150,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0"/>
-            <a:t> = residual capacity after rupture (FEM only)</a:t>
+            <a:t> = residual capacity after rupture</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -2115,7 +2160,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0"/>
-            <a:t> = modulus of elasticity of reinforcement (FEM only)</a:t>
+            <a:t> = modulus of elasticity of reinforcement</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -2125,7 +2170,48 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0"/>
-            <a:t> = cross-sectional area of reinforcement (FEM only)</a:t>
+            <a:t> = cross-sectional area of reinforcement</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Joint</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = model as slip element; mesh splits along line</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>kn</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint normal stiffness (blank = from soil E and size)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>ks</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint shear stiffness (blank = from soil G and size)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>Jred</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = reduce joint strength in SSRM (blank = Yes)</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="en-US" sz="1100" b="0"/>
@@ -2140,6 +2226,275 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>308428</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>172357</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>172356</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DA6D3C4-0920-BE4C-AFB2-D27825A644F5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12237357" y="571500"/>
+          <a:ext cx="3701143" cy="1995713"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Label</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = name used in error messages, summaries, and plots</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>(x1, y1), (x2, y2) </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t>= start and end of joint line</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>c</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint cohesion</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>phi</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint friction angle, degrees</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>c_res</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = residual joint cohesion (blank = same as c)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>phi_res</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = residual joint friction angle (blank = same as phi)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>dil</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint dilation angle, degrees (blank = 0)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>t_cut</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = tension cutoff (blank = 0)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>kn</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint normal stiffness (blank = from soil E and size)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>ks</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint shear stiffness (blank = from soil G and size)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>Jred</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = reduce joint strength in SSRM (blank = Yes)</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="0"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -2884,7 +3239,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="30">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -3028,10 +3383,10 @@
       </c>
       <c r="D17" s="1"/>
       <c r="F17" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G17" t="s">
-        <v>38</v>
+        <v>324</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
@@ -3039,10 +3394,10 @@
         <v>39</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G18" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D18"/>
     </row>
@@ -3051,10 +3406,10 @@
         <v>42</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G19" s="9" t="s">
-        <v>44</v>
+        <v>40</v>
+      </c>
+      <c r="G19" t="s">
+        <v>41</v>
       </c>
       <c r="D19"/>
     </row>
@@ -3063,10 +3418,10 @@
         <v>312</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D20"/>
     </row>
@@ -3075,10 +3430,10 @@
         <v>45</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="G21" t="s">
-        <v>50</v>
+        <v>46</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>47</v>
       </c>
       <c r="D21"/>
     </row>
@@ -3086,7 +3441,12 @@
       <c r="C22" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="F22" s="1"/>
+      <c r="F22" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G22" t="s">
+        <v>50</v>
+      </c>
       <c r="D22"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
@@ -3284,18 +3644,18 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A2:AD25"/>
+  <dimension ref="A2:AJ32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
     <col min="2" max="6" width="10.83203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="13.1640625" customWidth="1"/>
     <col min="10" max="14" width="10.83203125" style="1" customWidth="1"/>
-    <col min="18" max="20" width="10.83203125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="4.33203125" customWidth="1"/>
+    <col min="18" max="24" width="10.83203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="4.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>193</v>
       </c>
@@ -3356,17 +3716,33 @@
       <c r="T2" s="28" t="s">
         <v>256</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="U2" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="V2" s="28" t="s">
+        <v>320</v>
+      </c>
+      <c r="W2" s="28" t="s">
+        <v>321</v>
+      </c>
+      <c r="X2" s="28" t="s">
+        <v>322</v>
+      </c>
+      <c r="Z2" s="42"/>
+      <c r="AA2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AH2" t="s">
         <v>257</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AI2" t="s">
         <v>258</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AJ2" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -3377,11 +3753,11 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3" t="str">
-        <f t="shared" ref="H3:H22" si="0">IF($G3="","",IFERROR(VLOOKUP($G3,$AB$8:$AD$11,2,0),""))</f>
+        <f t="shared" ref="H3:H32" si="0">IF($G3="","",IFERROR(VLOOKUP($G3,$AH$8:$AJ$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I3" s="3" t="str">
-        <f t="shared" ref="I3:I22" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$AB$8:$AD$11,3,0),""))</f>
+        <f t="shared" ref="I3:I32" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$AH$8:$AJ$11,3,0),""))</f>
         <v/>
       </c>
       <c r="J3" s="3"/>
@@ -3395,17 +3771,25 @@
       <c r="R3" s="3"/>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
-      <c r="AB3" t="s">
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Z3" s="26"/>
+      <c r="AA3" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="AH3" t="s">
         <v>260</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AI3" t="s">
         <v>261</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="AJ3" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -3434,11 +3818,19 @@
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
-      <c r="AB4" t="s">
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Z4" s="29"/>
+      <c r="AA4" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="AH4" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -3467,11 +3859,15 @@
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
-      <c r="AB5" t="s">
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="AH5" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -3500,8 +3896,12 @@
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U6" s="3"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="3"/>
+      <c r="X6" s="3"/>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -3530,8 +3930,12 @@
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U7" s="3"/>
+      <c r="V7" s="3"/>
+      <c r="W7" s="3"/>
+      <c r="X7" s="3"/>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -3560,17 +3964,21 @@
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
       <c r="T8" s="3"/>
-      <c r="AB8" t="s">
+      <c r="U8" s="3"/>
+      <c r="V8" s="3"/>
+      <c r="W8" s="3"/>
+      <c r="X8" s="3"/>
+      <c r="AH8" t="s">
         <v>257</v>
       </c>
-      <c r="AC8" t="s">
+      <c r="AI8" t="s">
         <v>258</v>
       </c>
-      <c r="AD8" t="s">
+      <c r="AJ8" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -3599,17 +4007,21 @@
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
-      <c r="AB9" t="s">
+      <c r="U9" s="3"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="3"/>
+      <c r="X9" s="3"/>
+      <c r="AH9" t="s">
         <v>260</v>
       </c>
-      <c r="AC9" t="s">
+      <c r="AI9" t="s">
         <v>261</v>
       </c>
-      <c r="AD9" t="s">
+      <c r="AJ9" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -3638,17 +4050,21 @@
       <c r="R10" s="3"/>
       <c r="S10" s="3"/>
       <c r="T10" s="3"/>
-      <c r="AB10" t="s">
+      <c r="U10" s="3"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="3"/>
+      <c r="X10" s="3"/>
+      <c r="AH10" t="s">
         <v>263</v>
       </c>
-      <c r="AC10" t="s">
+      <c r="AI10" t="s">
         <v>261</v>
       </c>
-      <c r="AD10" t="s">
+      <c r="AJ10" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -3677,17 +4093,21 @@
       <c r="R11" s="3"/>
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
-      <c r="AB11" t="s">
+      <c r="U11" s="3"/>
+      <c r="V11" s="3"/>
+      <c r="W11" s="3"/>
+      <c r="X11" s="3"/>
+      <c r="AH11" t="s">
         <v>264</v>
       </c>
-      <c r="AC11" t="s">
+      <c r="AI11" t="s">
         <v>261</v>
       </c>
-      <c r="AD11" t="s">
+      <c r="AJ11" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -3716,8 +4136,12 @@
       <c r="R12" s="3"/>
       <c r="S12" s="3"/>
       <c r="T12" s="3"/>
-    </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U12" s="3"/>
+      <c r="V12" s="3"/>
+      <c r="W12" s="3"/>
+      <c r="X12" s="3"/>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -3746,8 +4170,12 @@
       <c r="R13" s="3"/>
       <c r="S13" s="3"/>
       <c r="T13" s="3"/>
-    </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U13" s="3"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="3"/>
+      <c r="X13" s="3"/>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -3776,8 +4204,12 @@
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U14" s="3"/>
+      <c r="V14" s="3"/>
+      <c r="W14" s="3"/>
+      <c r="X14" s="3"/>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -3806,8 +4238,12 @@
       <c r="R15" s="3"/>
       <c r="S15" s="3"/>
       <c r="T15" s="3"/>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U15" s="3"/>
+      <c r="V15" s="3"/>
+      <c r="W15" s="3"/>
+      <c r="X15" s="3"/>
+    </row>
+    <row r="16" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -3836,8 +4272,12 @@
       <c r="R16" s="3"/>
       <c r="S16" s="3"/>
       <c r="T16" s="3"/>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U16" s="3"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="3"/>
+      <c r="X16" s="3"/>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -3866,8 +4306,12 @@
       <c r="R17" s="3"/>
       <c r="S17" s="3"/>
       <c r="T17" s="3"/>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U17" s="3"/>
+      <c r="V17" s="3"/>
+      <c r="W17" s="3"/>
+      <c r="X17" s="3"/>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -3896,8 +4340,12 @@
       <c r="R18" s="3"/>
       <c r="S18" s="3"/>
       <c r="T18" s="3"/>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U18" s="3"/>
+      <c r="V18" s="3"/>
+      <c r="W18" s="3"/>
+      <c r="X18" s="3"/>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -3926,8 +4374,12 @@
       <c r="R19" s="3"/>
       <c r="S19" s="3"/>
       <c r="T19" s="3"/>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U19" s="3"/>
+      <c r="V19" s="3"/>
+      <c r="W19" s="3"/>
+      <c r="X19" s="3"/>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -3956,8 +4408,12 @@
       <c r="R20" s="3"/>
       <c r="S20" s="3"/>
       <c r="T20" s="3"/>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U20" s="3"/>
+      <c r="V20" s="3"/>
+      <c r="W20" s="3"/>
+      <c r="X20" s="3"/>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -3986,8 +4442,12 @@
       <c r="R21" s="3"/>
       <c r="S21" s="3"/>
       <c r="T21" s="3"/>
-    </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U21" s="3"/>
+      <c r="V21" s="3"/>
+      <c r="W21" s="3"/>
+      <c r="X21" s="3"/>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -4016,39 +4476,374 @@
       <c r="R22" s="3"/>
       <c r="S22" s="3"/>
       <c r="T22" s="3"/>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="V23" s="42"/>
-      <c r="W23" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
-      <c r="V24" s="26"/>
-      <c r="W24" s="9" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="K25" s="9"/>
-      <c r="L25" s="9"/>
-      <c r="V25" s="29"/>
-      <c r="W25" s="9" t="s">
-        <v>103</v>
-      </c>
+      <c r="U22" s="3"/>
+      <c r="V22" s="3"/>
+      <c r="W22" s="3"/>
+      <c r="X22" s="3"/>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A23" s="3">
+        <v>21</v>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I23" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="3"/>
+      <c r="Q23" s="3"/>
+      <c r="R23" s="3"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
+      <c r="U23" s="3"/>
+      <c r="V23" s="3"/>
+      <c r="W23" s="3"/>
+      <c r="X23" s="3"/>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A24" s="3">
+        <v>22</v>
+      </c>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I24" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+      <c r="P24" s="3"/>
+      <c r="Q24" s="3"/>
+      <c r="R24" s="3"/>
+      <c r="S24" s="3"/>
+      <c r="T24" s="3"/>
+      <c r="U24" s="3"/>
+      <c r="V24" s="3"/>
+      <c r="W24" s="3"/>
+      <c r="X24" s="3"/>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>23</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I25" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
+      <c r="R25" s="3"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
+      <c r="U25" s="3"/>
+      <c r="V25" s="3"/>
+      <c r="W25" s="3"/>
+      <c r="X25" s="3"/>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A26" s="3">
+        <v>24</v>
+      </c>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I26" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+      <c r="P26" s="3"/>
+      <c r="Q26" s="3"/>
+      <c r="R26" s="3"/>
+      <c r="S26" s="3"/>
+      <c r="T26" s="3"/>
+      <c r="U26" s="3"/>
+      <c r="V26" s="3"/>
+      <c r="W26" s="3"/>
+      <c r="X26" s="3"/>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A27" s="3">
+        <v>25</v>
+      </c>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I27" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+      <c r="P27" s="3"/>
+      <c r="Q27" s="3"/>
+      <c r="R27" s="3"/>
+      <c r="S27" s="3"/>
+      <c r="T27" s="3"/>
+      <c r="U27" s="3"/>
+      <c r="V27" s="3"/>
+      <c r="W27" s="3"/>
+      <c r="X27" s="3"/>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A28" s="3">
+        <v>26</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I28" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="3"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+      <c r="R28" s="3"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="3"/>
+      <c r="U28" s="3"/>
+      <c r="V28" s="3"/>
+      <c r="W28" s="3"/>
+      <c r="X28" s="3"/>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A29" s="3">
+        <v>27</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I29" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+      <c r="P29" s="3"/>
+      <c r="Q29" s="3"/>
+      <c r="R29" s="3"/>
+      <c r="S29" s="3"/>
+      <c r="T29" s="3"/>
+      <c r="U29" s="3"/>
+      <c r="V29" s="3"/>
+      <c r="W29" s="3"/>
+      <c r="X29" s="3"/>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A30" s="3">
+        <v>28</v>
+      </c>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I30" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+      <c r="P30" s="3"/>
+      <c r="Q30" s="3"/>
+      <c r="R30" s="3"/>
+      <c r="S30" s="3"/>
+      <c r="T30" s="3"/>
+      <c r="U30" s="3"/>
+      <c r="V30" s="3"/>
+      <c r="W30" s="3"/>
+      <c r="X30" s="3"/>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A31" s="3">
+        <v>29</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I31" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="3"/>
+      <c r="N31" s="3"/>
+      <c r="O31" s="3"/>
+      <c r="P31" s="3"/>
+      <c r="Q31" s="3"/>
+      <c r="R31" s="3"/>
+      <c r="S31" s="3"/>
+      <c r="T31" s="3"/>
+      <c r="U31" s="3"/>
+      <c r="V31" s="3"/>
+      <c r="W31" s="3"/>
+      <c r="X31" s="3"/>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A32" s="3">
+        <v>30</v>
+      </c>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I32" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="3"/>
+      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
+      <c r="P32" s="3"/>
+      <c r="Q32" s="3"/>
+      <c r="R32" s="3"/>
+      <c r="S32" s="3"/>
+      <c r="T32" s="3"/>
+      <c r="U32" s="3"/>
+      <c r="V32" s="3"/>
+      <c r="W32" s="3"/>
+      <c r="X32" s="3"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G22" xr:uid="{00000000-0002-0000-0900-000000000000}">
-      <formula1>$AB$2:$AB$5</formula1>
+  <conditionalFormatting sqref="K3:L32">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>$U3="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V3:X32">
+    <cfRule type="expression" dxfId="0" priority="4">
+      <formula>$U3&lt;&gt;"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G32" xr:uid="{00000000-0002-0000-0900-000000000000}">
+      <formula1>$AH$2:$AH$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H22" xr:uid="{00000000-0002-0000-0900-000001000000}">
-      <formula1>$AC$2:$AC$3</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H32" xr:uid="{00000000-0002-0000-0900-000001000000}">
+      <formula1>$AI$2:$AI$3</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I22" xr:uid="{00000000-0002-0000-0900-000002000000}">
-      <formula1>$AD$2:$AD$3</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I32" xr:uid="{00000000-0002-0000-0900-000002000000}">
+      <formula1>$AJ$2:$AJ$3</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U3:U32 X3:X32" xr:uid="{8FB27197-C456-2D4D-8100-E78D5059F972}">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4057,6 +4852,1028 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C676759-96FB-7F49-B49A-BD8077ECE53B}">
+  <dimension ref="A2:R52"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
+    <col min="2" max="15" width="10.83203125" style="1" customWidth="1"/>
+    <col min="16" max="16" width="4.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="G2" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="H2" s="28" t="s">
+        <v>323</v>
+      </c>
+      <c r="I2" s="28" t="s">
+        <v>326</v>
+      </c>
+      <c r="J2" s="28" t="s">
+        <v>327</v>
+      </c>
+      <c r="K2" s="28" t="s">
+        <v>328</v>
+      </c>
+      <c r="L2" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="M2" s="28" t="s">
+        <v>320</v>
+      </c>
+      <c r="N2" s="28" t="s">
+        <v>321</v>
+      </c>
+      <c r="O2" s="28" t="s">
+        <v>322</v>
+      </c>
+      <c r="Q2" s="29"/>
+      <c r="R2" s="9" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A5" s="3">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A6" s="3">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A10" s="3">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A12" s="3">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A13" s="3">
+        <v>11</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
+      <c r="O13" s="3"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A14" s="3">
+        <v>12</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="N14" s="3"/>
+      <c r="O14" s="3"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A15" s="3">
+        <v>13</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="3"/>
+      <c r="O15" s="3"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A16" s="3">
+        <v>14</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="3"/>
+      <c r="N16" s="3"/>
+      <c r="O16" s="3"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A17" s="3">
+        <v>15</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="3"/>
+      <c r="O17" s="3"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A18" s="3">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3"/>
+      <c r="N18" s="3"/>
+      <c r="O18" s="3"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A19" s="3">
+        <v>17</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+      <c r="O19" s="3"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A20" s="3">
+        <v>18</v>
+      </c>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="3"/>
+      <c r="O20" s="3"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A21" s="3">
+        <v>19</v>
+      </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="3"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A22" s="3">
+        <v>20</v>
+      </c>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
+      <c r="O22" s="3"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A23" s="3">
+        <v>21</v>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A24" s="3">
+        <v>22</v>
+      </c>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>23</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A26" s="3">
+        <v>24</v>
+      </c>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A27" s="3">
+        <v>25</v>
+      </c>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A28" s="3">
+        <v>26</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="3"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A29" s="3">
+        <v>27</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A30" s="3">
+        <v>28</v>
+      </c>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A31" s="3">
+        <v>29</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="3"/>
+      <c r="N31" s="3"/>
+      <c r="O31" s="3"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A32" s="3">
+        <v>30</v>
+      </c>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="3"/>
+      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A33" s="3">
+        <v>31</v>
+      </c>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
+      <c r="N33" s="3"/>
+      <c r="O33" s="3"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A34" s="3">
+        <v>32</v>
+      </c>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
+      <c r="N34" s="3"/>
+      <c r="O34" s="3"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A35" s="3">
+        <v>33</v>
+      </c>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+      <c r="K35" s="3"/>
+      <c r="L35" s="3"/>
+      <c r="M35" s="3"/>
+      <c r="N35" s="3"/>
+      <c r="O35" s="3"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A36" s="3">
+        <v>34</v>
+      </c>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="3"/>
+      <c r="N36" s="3"/>
+      <c r="O36" s="3"/>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A37" s="3">
+        <v>35</v>
+      </c>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3"/>
+      <c r="M37" s="3"/>
+      <c r="N37" s="3"/>
+      <c r="O37" s="3"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A38" s="3">
+        <v>36</v>
+      </c>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
+      <c r="L38" s="3"/>
+      <c r="M38" s="3"/>
+      <c r="N38" s="3"/>
+      <c r="O38" s="3"/>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A39" s="3">
+        <v>37</v>
+      </c>
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+      <c r="K39" s="3"/>
+      <c r="L39" s="3"/>
+      <c r="M39" s="3"/>
+      <c r="N39" s="3"/>
+      <c r="O39" s="3"/>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A40" s="3">
+        <v>38</v>
+      </c>
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="3"/>
+      <c r="L40" s="3"/>
+      <c r="M40" s="3"/>
+      <c r="N40" s="3"/>
+      <c r="O40" s="3"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A41" s="3">
+        <v>39</v>
+      </c>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+      <c r="I41" s="3"/>
+      <c r="J41" s="3"/>
+      <c r="K41" s="3"/>
+      <c r="L41" s="3"/>
+      <c r="M41" s="3"/>
+      <c r="N41" s="3"/>
+      <c r="O41" s="3"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A42" s="3">
+        <v>40</v>
+      </c>
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
+      <c r="L42" s="3"/>
+      <c r="M42" s="3"/>
+      <c r="N42" s="3"/>
+      <c r="O42" s="3"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A43" s="3">
+        <v>41</v>
+      </c>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="3"/>
+      <c r="L43" s="3"/>
+      <c r="M43" s="3"/>
+      <c r="N43" s="3"/>
+      <c r="O43" s="3"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A44" s="3">
+        <v>42</v>
+      </c>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="3"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="3"/>
+      <c r="L44" s="3"/>
+      <c r="M44" s="3"/>
+      <c r="N44" s="3"/>
+      <c r="O44" s="3"/>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A45" s="3">
+        <v>43</v>
+      </c>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
+      <c r="N45" s="3"/>
+      <c r="O45" s="3"/>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A46" s="3">
+        <v>44</v>
+      </c>
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="3"/>
+      <c r="K46" s="3"/>
+      <c r="L46" s="3"/>
+      <c r="M46" s="3"/>
+      <c r="N46" s="3"/>
+      <c r="O46" s="3"/>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <v>45</v>
+      </c>
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="3"/>
+      <c r="M47" s="3"/>
+      <c r="N47" s="3"/>
+      <c r="O47" s="3"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A48" s="3">
+        <v>46</v>
+      </c>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="3"/>
+      <c r="L48" s="3"/>
+      <c r="M48" s="3"/>
+      <c r="N48" s="3"/>
+      <c r="O48" s="3"/>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A49" s="3">
+        <v>47</v>
+      </c>
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
+      <c r="K49" s="3"/>
+      <c r="L49" s="3"/>
+      <c r="M49" s="3"/>
+      <c r="N49" s="3"/>
+      <c r="O49" s="3"/>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A50" s="3">
+        <v>48</v>
+      </c>
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="3"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="3"/>
+      <c r="N50" s="3"/>
+      <c r="O50" s="3"/>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A51" s="3">
+        <v>49</v>
+      </c>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
+      <c r="N51" s="3"/>
+      <c r="O51" s="3"/>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A52" s="3">
+        <v>50</v>
+      </c>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+      <c r="J52" s="3"/>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+      <c r="M52" s="3"/>
+      <c r="N52" s="3"/>
+      <c r="O52" s="3"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O3:O52" xr:uid="{D1121F3C-F660-0E46-8AEB-8C1F95C55489}">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A2:AA17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4386,7 +6203,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A2:F22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4621,7 +6438,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="B2:U24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -5067,7 +6884,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="B2:U24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -5481,7 +7298,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="B2:J100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -8422,83 +10239,83 @@
     <mergeCell ref="C9:Z9"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:K52 AB11:AF52">
-    <cfRule type="expression" dxfId="34" priority="6">
+    <cfRule type="expression" dxfId="36" priority="6">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="7">
+    <cfRule type="expression" dxfId="35" priority="7">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11:L52 O11:R52">
-    <cfRule type="expression" dxfId="32" priority="19">
+    <cfRule type="expression" dxfId="34" priority="19">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="31" priority="8">
+    <cfRule type="expression" dxfId="33" priority="8">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="30" priority="9">
+    <cfRule type="expression" dxfId="32" priority="9">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:K52">
-    <cfRule type="expression" dxfId="29" priority="10">
+    <cfRule type="expression" dxfId="31" priority="10">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P11:P52">
-    <cfRule type="expression" dxfId="28" priority="13">
+    <cfRule type="expression" dxfId="30" priority="13">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="27" priority="23">
+    <cfRule type="expression" dxfId="29" priority="23">
       <formula>$E11="cp"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="24">
+    <cfRule type="expression" dxfId="28" priority="24">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S11:V52">
-    <cfRule type="expression" dxfId="25" priority="11">
+    <cfRule type="expression" dxfId="27" priority="11">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W11:Z52">
-    <cfRule type="expression" dxfId="24" priority="12">
+    <cfRule type="expression" dxfId="26" priority="12">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB11:AF52">
-    <cfRule type="expression" dxfId="23" priority="21">
+    <cfRule type="expression" dxfId="25" priority="21">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC11:AC52">
-    <cfRule type="expression" dxfId="22" priority="14">
+    <cfRule type="expression" dxfId="24" priority="14">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD11:AD52">
-    <cfRule type="expression" dxfId="21" priority="15">
+    <cfRule type="expression" dxfId="23" priority="15">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE11:AF52">
-    <cfRule type="expression" dxfId="20" priority="16">
+    <cfRule type="expression" dxfId="22" priority="16">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="19" priority="17">
+    <cfRule type="expression" dxfId="21" priority="17">
       <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AM11:AO52">
-    <cfRule type="expression" dxfId="18" priority="1">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>$AJ11="lf"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8548,7 +10365,7 @@
         <v>145</v>
       </c>
       <c r="B2" s="3">
-        <v>0.0</v>
+        <v>182.0</v>
       </c>
       <c r="D2" s="24" t="s">
         <v>146</v>
@@ -11274,83 +13091,83 @@
     <mergeCell ref="V7:W7"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
-    <cfRule type="expression" dxfId="17" priority="1">
+    <cfRule type="expression" dxfId="19" priority="1">
       <formula>AND($B$5&lt;&gt;"",$B$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6 D7:E7">
-    <cfRule type="expression" dxfId="16" priority="2">
+    <cfRule type="expression" dxfId="18" priority="2">
       <formula>AND($E$5&lt;&gt;"",$E$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6 G7:H7">
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="17" priority="3">
       <formula>AND($H$5&lt;&gt;"",$H$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6 J7:K7">
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="16" priority="4">
       <formula>AND($K$5&lt;&gt;"",$K$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N6 M7:N7">
-    <cfRule type="expression" dxfId="13" priority="5">
+    <cfRule type="expression" dxfId="15" priority="5">
       <formula>AND($N$5&lt;&gt;"",$N$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q6 P7:Q7">
-    <cfRule type="expression" dxfId="12" priority="6">
+    <cfRule type="expression" dxfId="14" priority="6">
       <formula>AND($Q$5&lt;&gt;"",$Q$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T6 S7:T7">
-    <cfRule type="expression" dxfId="11" priority="7">
+    <cfRule type="expression" dxfId="13" priority="7">
       <formula>AND($T$5&lt;&gt;"",$T$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W6 V7:W7">
-    <cfRule type="expression" dxfId="10" priority="8">
+    <cfRule type="expression" dxfId="12" priority="8">
       <formula>AND($W$5&lt;&gt;"",$W$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z6 Y7:Z7">
-    <cfRule type="expression" dxfId="9" priority="9">
+    <cfRule type="expression" dxfId="11" priority="9">
       <formula>AND($Z$5&lt;&gt;"",$Z$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC6 AB7:AC7">
-    <cfRule type="expression" dxfId="8" priority="10">
+    <cfRule type="expression" dxfId="10" priority="10">
       <formula>AND($AC$5&lt;&gt;"",$AC$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF6 AE7:AF7">
-    <cfRule type="expression" dxfId="7" priority="11">
+    <cfRule type="expression" dxfId="9" priority="11">
       <formula>AND($AF$5&lt;&gt;"",$AF$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI6 AH7:AI7">
-    <cfRule type="expression" dxfId="6" priority="12">
+    <cfRule type="expression" dxfId="8" priority="12">
       <formula>AND($AI$5&lt;&gt;"",$AI$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL6 AK7:AL7">
-    <cfRule type="expression" dxfId="5" priority="13">
+    <cfRule type="expression" dxfId="7" priority="13">
       <formula>AND($AL$5&lt;&gt;"",$AL$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO6 AN7:AO7">
-    <cfRule type="expression" dxfId="4" priority="14">
+    <cfRule type="expression" dxfId="6" priority="14">
       <formula>AND($AO$5&lt;&gt;"",$AO$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AR6 AQ7:AR7">
-    <cfRule type="expression" dxfId="3" priority="15">
+    <cfRule type="expression" dxfId="5" priority="15">
       <formula>AND($AR$5&lt;&gt;"",$AR$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5 E5 H5 K5 N5 Q5 T5 W5 Z5 AC5 AF5 AI5 AL5 AO5 AR5" xr:uid="{00000000-0002-0000-0300-000000000000}">
-      <formula1>"material,ssr reduce,ssr hold,ssr elastic,refine"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5 E5 H5 K5 N5 Q5 T5 W5 Z5 AC5 AF5 AI5 AL5 AO5 AR5" xr:uid="{2C58C22E-BB25-6145-9297-FDBC71F3461D}">
+      <formula1>"material,ssr reduce,ssr hold,ssr elastic,refine,joints"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11868,17 +13685,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E42">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:G42">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>OR($D3="Depth",$D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>OR($D3="Depth",$D3="Intercept")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>